<commit_message>
Improve recovery status logic and update visualizations
Enhanced the disease metrics calculation in forecast.R to use both recovery trend and payback for robust recovery detection. Updated visualization scripts to include 'Status' and improved labeling for periods. Changed legend label in best model plot to 'Composite index'. Updated related data and figure files to reflect these changes.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig3.xlsx
+++ b/Outcome/Publish/figure_data/fig3.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
   <si>
     <t xml:space="preserve">Group</t>
   </si>
@@ -207,6 +207,9 @@
     <t xml:space="preserve">StartDate</t>
   </si>
   <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
     <t xml:space="preserve">type</t>
   </si>
   <si>
@@ -216,94 +219,107 @@
     <t xml:space="preserve">Period</t>
   </si>
   <si>
+    <t xml:space="preserve">Debt Repaid</t>
+  </si>
+  <si>
     <t xml:space="preserve">Recovery</t>
   </si>
   <si>
-    <t xml:space="preserve">34 months</t>
+    <t xml:space="preserve">34m</t>
   </si>
   <si>
     <t xml:space="preserve">Balance</t>
   </si>
   <si>
-    <t xml:space="preserve">61 months</t>
+    <t xml:space="preserve">61m</t>
   </si>
   <si>
-    <t xml:space="preserve">43 months</t>
+    <t xml:space="preserve">Recovered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43m</t>
   </si>
   <si>
     <t xml:space="preserve">Not balanced</t>
   </si>
   <si>
+    <t xml:space="preserve">Suppressed</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not recovered</t>
   </si>
   <si>
-    <t xml:space="preserve">56 months</t>
+    <t xml:space="preserve">58m</t>
   </si>
   <si>
-    <t xml:space="preserve">35 months</t>
+    <t xml:space="preserve">35m</t>
   </si>
   <si>
-    <t xml:space="preserve">27 months</t>
+    <t xml:space="preserve">No Deficit</t>
   </si>
   <si>
-    <t xml:space="preserve">32 months</t>
+    <t xml:space="preserve">No deficit</t>
   </si>
   <si>
-    <t xml:space="preserve">33 months</t>
+    <t xml:space="preserve">27m</t>
   </si>
   <si>
-    <t xml:space="preserve">7 months</t>
+    <t xml:space="preserve">32m</t>
   </si>
   <si>
-    <t xml:space="preserve">41 months</t>
+    <t xml:space="preserve">28m</t>
   </si>
   <si>
-    <t xml:space="preserve">4 months</t>
+    <t xml:space="preserve">33m</t>
   </si>
   <si>
-    <t xml:space="preserve">6 months</t>
+    <t xml:space="preserve">41m</t>
   </si>
   <si>
-    <t xml:space="preserve">9 months</t>
+    <t xml:space="preserve">5m</t>
   </si>
   <si>
-    <t xml:space="preserve">29 months</t>
+    <t xml:space="preserve">6m</t>
   </si>
   <si>
-    <t xml:space="preserve">36 months</t>
+    <t xml:space="preserve">9m</t>
   </si>
   <si>
-    <t xml:space="preserve">30 months</t>
+    <t xml:space="preserve">29m</t>
   </si>
   <si>
-    <t xml:space="preserve">54 months</t>
+    <t xml:space="preserve">36m</t>
   </si>
   <si>
-    <t xml:space="preserve">0 months</t>
+    <t xml:space="preserve">31m</t>
   </si>
   <si>
-    <t xml:space="preserve">52 months</t>
+    <t xml:space="preserve">30m</t>
   </si>
   <si>
-    <t xml:space="preserve">40 months</t>
+    <t xml:space="preserve">54m</t>
   </si>
   <si>
-    <t xml:space="preserve">51 months</t>
+    <t xml:space="preserve">46m</t>
   </si>
   <si>
-    <t xml:space="preserve">44 months</t>
+    <t xml:space="preserve">52m</t>
   </si>
   <si>
-    <t xml:space="preserve">28 months</t>
+    <t xml:space="preserve">56m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">48m</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -340,7 +356,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -47615,6 +47631,9 @@
       <c r="E1" t="s">
         <v>58</v>
       </c>
+      <c r="F1" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -47624,13 +47643,16 @@
         <v>43831</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" s="1" t="n">
         <v>44866</v>
       </c>
-      <c r="E2" t="s">
-        <v>60</v>
+      <c r="F2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="3">
@@ -47641,13 +47663,16 @@
         <v>43831</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D3" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="1" t="n">
         <v>45689</v>
       </c>
-      <c r="E3" t="s">
-        <v>62</v>
+      <c r="F3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="4">
@@ -47658,13 +47683,16 @@
         <v>43831</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D4" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="1" t="n">
         <v>45139</v>
       </c>
-      <c r="E4" t="s">
-        <v>63</v>
+      <c r="F4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="5">
@@ -47675,13 +47703,16 @@
         <v>43831</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D5" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E5" t="s">
-        <v>64</v>
+      <c r="F5" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="6">
@@ -47692,13 +47723,16 @@
         <v>43831</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D6" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E6" t="s">
-        <v>65</v>
+      <c r="F6" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="7">
@@ -47709,13 +47743,16 @@
         <v>43831</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="D7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E7" t="s">
-        <v>64</v>
+      <c r="F7" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="8">
@@ -47726,13 +47763,16 @@
         <v>43831</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>45536</v>
-      </c>
-      <c r="E8" t="s">
-        <v>66</v>
+        <v>65</v>
+      </c>
+      <c r="D8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>45597</v>
+      </c>
+      <c r="F8" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="9">
@@ -47743,13 +47783,16 @@
         <v>43831</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
-      </c>
-      <c r="D9" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E9" t="s">
-        <v>64</v>
+      <c r="F9" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="10">
@@ -47760,13 +47803,16 @@
         <v>43831</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
-      </c>
-      <c r="D10" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" s="1" t="n">
         <v>45689</v>
       </c>
-      <c r="E10" t="s">
-        <v>62</v>
+      <c r="F10" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="11">
@@ -47777,13 +47823,16 @@
         <v>43831</v>
       </c>
       <c r="C11" t="s">
-        <v>61</v>
-      </c>
-      <c r="D11" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E11" t="s">
-        <v>64</v>
+      <c r="F11" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="12">
@@ -47794,13 +47843,16 @@
         <v>43831</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
-      </c>
-      <c r="D12" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>61</v>
+      </c>
+      <c r="E12" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E12" t="s">
-        <v>65</v>
+      <c r="F12" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="13">
@@ -47811,13 +47863,16 @@
         <v>43831</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="D13" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E13" t="s">
-        <v>64</v>
+      <c r="F13" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="14">
@@ -47828,13 +47883,16 @@
         <v>43831</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
-      </c>
-      <c r="D14" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="1" t="n">
         <v>44896</v>
       </c>
-      <c r="E14" t="s">
-        <v>67</v>
+      <c r="F14" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="15">
@@ -47845,13 +47903,16 @@
         <v>43831</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E15" t="s">
-        <v>64</v>
+      <c r="F15" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="16">
@@ -47862,13 +47923,16 @@
         <v>43831</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="D16" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E16" t="s">
-        <v>65</v>
+      <c r="F16" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="17">
@@ -47879,13 +47943,16 @@
         <v>43831</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
-      </c>
-      <c r="D17" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="D17" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E17" t="s">
-        <v>64</v>
+      <c r="F17" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="18">
@@ -47896,13 +47963,16 @@
         <v>43831</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D18" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" s="1" t="n">
         <v>44652</v>
       </c>
-      <c r="E18" t="s">
-        <v>68</v>
+      <c r="F18" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="19">
@@ -47913,13 +47983,16 @@
         <v>43831</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
-      </c>
-      <c r="D19" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D19" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="1" t="n">
         <v>44805</v>
       </c>
-      <c r="E19" t="s">
-        <v>69</v>
+      <c r="F19" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="20">
@@ -47930,13 +48003,16 @@
         <v>43831</v>
       </c>
       <c r="C20" t="s">
-        <v>59</v>
-      </c>
-      <c r="D20" s="1" t="n">
-        <v>44652</v>
-      </c>
-      <c r="E20" t="s">
-        <v>68</v>
+        <v>60</v>
+      </c>
+      <c r="D20" t="s">
+        <v>61</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>44682</v>
+      </c>
+      <c r="F20" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="21">
@@ -47947,13 +48023,16 @@
         <v>43831</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="1" t="n">
         <v>44835</v>
       </c>
-      <c r="E21" t="s">
-        <v>70</v>
+      <c r="F21" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="22">
@@ -47964,13 +48043,16 @@
         <v>43831</v>
       </c>
       <c r="C22" t="s">
-        <v>59</v>
-      </c>
-      <c r="D22" s="1" t="n">
-        <v>44044</v>
-      </c>
-      <c r="E22" t="s">
-        <v>71</v>
+        <v>60</v>
+      </c>
+      <c r="D22" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>44682</v>
+      </c>
+      <c r="F22" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="23">
@@ -47981,13 +48063,16 @@
         <v>43831</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
-      </c>
-      <c r="D23" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D23" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="1" t="n">
         <v>45078</v>
       </c>
-      <c r="E23" t="s">
-        <v>72</v>
+      <c r="F23" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="24">
@@ -47998,13 +48083,16 @@
         <v>43831</v>
       </c>
       <c r="C24" t="s">
-        <v>59</v>
-      </c>
-      <c r="D24" s="1" t="n">
-        <v>43952</v>
-      </c>
-      <c r="E24" t="s">
-        <v>73</v>
+        <v>60</v>
+      </c>
+      <c r="D24" t="s">
+        <v>61</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>43983</v>
+      </c>
+      <c r="F24" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="25">
@@ -48015,13 +48103,16 @@
         <v>43831</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D25" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" s="1" t="n">
         <v>44013</v>
       </c>
-      <c r="E25" t="s">
-        <v>74</v>
+      <c r="F25" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="26">
@@ -48032,13 +48123,16 @@
         <v>43831</v>
       </c>
       <c r="C26" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D26" t="s">
+        <v>61</v>
+      </c>
+      <c r="E26" s="1" t="n">
         <v>44105</v>
       </c>
-      <c r="E26" t="s">
-        <v>75</v>
+      <c r="F26" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="27">
@@ -48049,13 +48143,16 @@
         <v>43831</v>
       </c>
       <c r="C27" t="s">
-        <v>61</v>
-      </c>
-      <c r="D27" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D27" t="s">
+        <v>63</v>
+      </c>
+      <c r="E27" s="1" t="n">
         <v>44805</v>
       </c>
-      <c r="E27" t="s">
-        <v>69</v>
+      <c r="F27" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="28">
@@ -48066,13 +48163,16 @@
         <v>43831</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
-      </c>
-      <c r="D28" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D28" t="s">
+        <v>61</v>
+      </c>
+      <c r="E28" s="1" t="n">
         <v>44713</v>
       </c>
-      <c r="E28" t="s">
-        <v>76</v>
+      <c r="F28" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="29">
@@ -48083,13 +48183,16 @@
         <v>43831</v>
       </c>
       <c r="C29" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D29" t="s">
+        <v>63</v>
+      </c>
+      <c r="E29" s="1" t="n">
         <v>44927</v>
       </c>
-      <c r="E29" t="s">
-        <v>77</v>
+      <c r="F29" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="30">
@@ -48100,13 +48203,16 @@
         <v>43831</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
-      </c>
-      <c r="D30" s="1" t="n">
-        <v>44713</v>
-      </c>
-      <c r="E30" t="s">
-        <v>76</v>
+        <v>65</v>
+      </c>
+      <c r="D30" t="s">
+        <v>61</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>44774</v>
+      </c>
+      <c r="F30" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="31">
@@ -48117,13 +48223,16 @@
         <v>43831</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
-      </c>
-      <c r="D31" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D31" t="s">
+        <v>63</v>
+      </c>
+      <c r="E31" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E31" t="s">
-        <v>64</v>
+      <c r="F31" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="32">
@@ -48134,13 +48243,16 @@
         <v>43831</v>
       </c>
       <c r="C32" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D32" t="s">
+        <v>61</v>
+      </c>
+      <c r="E32" s="1" t="n">
         <v>44743</v>
       </c>
-      <c r="E32" t="s">
-        <v>78</v>
+      <c r="F32" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="33">
@@ -48151,13 +48263,16 @@
         <v>43831</v>
       </c>
       <c r="C33" t="s">
-        <v>61</v>
-      </c>
-      <c r="D33" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D33" t="s">
+        <v>63</v>
+      </c>
+      <c r="E33" s="1" t="n">
         <v>45474</v>
       </c>
-      <c r="E33" t="s">
-        <v>79</v>
+      <c r="F33" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="34">
@@ -48168,13 +48283,16 @@
         <v>43831</v>
       </c>
       <c r="C34" t="s">
-        <v>59</v>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>43831</v>
-      </c>
-      <c r="E34" t="s">
-        <v>80</v>
+        <v>65</v>
+      </c>
+      <c r="D34" t="s">
+        <v>61</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>45231</v>
+      </c>
+      <c r="F34" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="35">
@@ -48185,13 +48303,16 @@
         <v>43831</v>
       </c>
       <c r="C35" t="s">
-        <v>61</v>
-      </c>
-      <c r="D35" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D35" t="s">
+        <v>63</v>
+      </c>
+      <c r="E35" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E35" t="s">
-        <v>64</v>
+      <c r="F35" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="36">
@@ -48202,13 +48323,16 @@
         <v>43831</v>
       </c>
       <c r="C36" t="s">
-        <v>59</v>
-      </c>
-      <c r="D36" s="1" t="n">
-        <v>44866</v>
-      </c>
-      <c r="E36" t="s">
         <v>60</v>
+      </c>
+      <c r="D36" t="s">
+        <v>61</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>44927</v>
+      </c>
+      <c r="F36" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="37">
@@ -48219,13 +48343,16 @@
         <v>43831</v>
       </c>
       <c r="C37" t="s">
-        <v>61</v>
-      </c>
-      <c r="D37" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D37" t="s">
+        <v>63</v>
+      </c>
+      <c r="E37" s="1" t="n">
         <v>45689</v>
       </c>
-      <c r="E37" t="s">
-        <v>62</v>
+      <c r="F37" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="38">
@@ -48236,13 +48363,16 @@
         <v>43831</v>
       </c>
       <c r="C38" t="s">
-        <v>59</v>
-      </c>
-      <c r="D38" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="D38" t="s">
+        <v>61</v>
+      </c>
+      <c r="E38" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E38" t="s">
-        <v>65</v>
+      <c r="F38" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="39">
@@ -48253,13 +48383,16 @@
         <v>43831</v>
       </c>
       <c r="C39" t="s">
-        <v>61</v>
-      </c>
-      <c r="D39" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="D39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E39" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E39" t="s">
-        <v>64</v>
+      <c r="F39" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="40">
@@ -48270,13 +48403,16 @@
         <v>43831</v>
       </c>
       <c r="C40" t="s">
-        <v>59</v>
-      </c>
-      <c r="D40" s="1" t="n">
-        <v>44927</v>
-      </c>
-      <c r="E40" t="s">
-        <v>77</v>
+        <v>60</v>
+      </c>
+      <c r="D40" t="s">
+        <v>61</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>45078</v>
+      </c>
+      <c r="F40" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="41">
@@ -48287,13 +48423,16 @@
         <v>43831</v>
       </c>
       <c r="C41" t="s">
-        <v>61</v>
-      </c>
-      <c r="D41" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D41" t="s">
+        <v>63</v>
+      </c>
+      <c r="E41" s="1" t="n">
         <v>45413</v>
       </c>
-      <c r="E41" t="s">
-        <v>81</v>
+      <c r="F41" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="42">
@@ -48304,13 +48443,16 @@
         <v>43831</v>
       </c>
       <c r="C42" t="s">
-        <v>59</v>
-      </c>
-      <c r="D42" s="1" t="n">
-        <v>45047</v>
-      </c>
-      <c r="E42" t="s">
-        <v>82</v>
+        <v>60</v>
+      </c>
+      <c r="D42" t="s">
+        <v>61</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>45139</v>
+      </c>
+      <c r="F42" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="43">
@@ -48321,13 +48463,16 @@
         <v>43831</v>
       </c>
       <c r="C43" t="s">
-        <v>61</v>
-      </c>
-      <c r="D43" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D43" t="s">
+        <v>63</v>
+      </c>
+      <c r="E43" s="1" t="n">
         <v>45536</v>
       </c>
-      <c r="E43" t="s">
-        <v>66</v>
+      <c r="F43" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="44">
@@ -48338,13 +48483,16 @@
         <v>43831</v>
       </c>
       <c r="C44" t="s">
-        <v>59</v>
-      </c>
-      <c r="D44" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D44" t="s">
+        <v>61</v>
+      </c>
+      <c r="E44" s="1" t="n">
         <v>44927</v>
       </c>
-      <c r="E44" t="s">
-        <v>77</v>
+      <c r="F44" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="45">
@@ -48355,13 +48503,16 @@
         <v>43831</v>
       </c>
       <c r="C45" t="s">
-        <v>61</v>
-      </c>
-      <c r="D45" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D45" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45" s="1" t="n">
         <v>45383</v>
       </c>
-      <c r="E45" t="s">
-        <v>83</v>
+      <c r="F45" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="46">
@@ -48372,13 +48523,16 @@
         <v>43831</v>
       </c>
       <c r="C46" t="s">
-        <v>59</v>
-      </c>
-      <c r="D46" s="1" t="n">
-        <v>45170</v>
-      </c>
-      <c r="E46" t="s">
-        <v>84</v>
+        <v>65</v>
+      </c>
+      <c r="D46" t="s">
+        <v>61</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>45292</v>
+      </c>
+      <c r="F46" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="47">
@@ -48389,13 +48543,16 @@
         <v>43831</v>
       </c>
       <c r="C47" t="s">
-        <v>61</v>
-      </c>
-      <c r="D47" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D47" t="s">
+        <v>63</v>
+      </c>
+      <c r="E47" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="E47" t="s">
-        <v>64</v>
+      <c r="F47" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="48">
@@ -48406,13 +48563,16 @@
         <v>43831</v>
       </c>
       <c r="C48" t="s">
-        <v>59</v>
-      </c>
-      <c r="D48" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D48" t="s">
+        <v>61</v>
+      </c>
+      <c r="E48" s="1" t="n">
         <v>44682</v>
       </c>
-      <c r="E48" t="s">
-        <v>85</v>
+      <c r="F48" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="49">
@@ -48423,13 +48583,16 @@
         <v>43831</v>
       </c>
       <c r="C49" t="s">
-        <v>61</v>
-      </c>
-      <c r="D49" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="D49" t="s">
+        <v>63</v>
+      </c>
+      <c r="E49" s="1" t="n">
         <v>44866</v>
       </c>
-      <c r="E49" t="s">
-        <v>60</v>
+      <c r="F49" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update figure data and improve visualization scripts
Updated figures (fig3, fig5, fig6) and their associated data files. Improved calculation of recovery and balance periods in 5_b_visualization.R, clarified axis labels and variable usage in 7_a_suppression.R and 8_a_recovery.R, and fixed the baseline vertical line reference in forecast.R to use the correct start date.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig3.xlsx
+++ b/Outcome/Publish/figure_data/fig3.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t xml:space="preserve">Group</t>
   </si>
@@ -225,19 +225,19 @@
     <t xml:space="preserve">Recovery</t>
   </si>
   <si>
-    <t xml:space="preserve">34m</t>
+    <t xml:space="preserve">31m</t>
   </si>
   <si>
     <t xml:space="preserve">Balance</t>
   </si>
   <si>
-    <t xml:space="preserve">61m</t>
+    <t xml:space="preserve">58m</t>
   </si>
   <si>
     <t xml:space="preserve">Recovered</t>
   </si>
   <si>
-    <t xml:space="preserve">43m</t>
+    <t xml:space="preserve">41m</t>
   </si>
   <si>
     <t xml:space="preserve">Not balanced</t>
@@ -249,10 +249,10 @@
     <t xml:space="preserve">Not recovered</t>
   </si>
   <si>
-    <t xml:space="preserve">58m</t>
+    <t xml:space="preserve">61m</t>
   </si>
   <si>
-    <t xml:space="preserve">35m</t>
+    <t xml:space="preserve">34m</t>
   </si>
   <si>
     <t xml:space="preserve">No Deficit</t>
@@ -261,37 +261,40 @@
     <t xml:space="preserve">No deficit</t>
   </si>
   <si>
+    <t xml:space="preserve">22m</t>
+  </si>
+  <si>
     <t xml:space="preserve">27m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9m</t>
   </si>
   <si>
     <t xml:space="preserve">32m</t>
   </si>
   <si>
-    <t xml:space="preserve">28m</t>
+    <t xml:space="preserve">11m</t>
   </si>
   <si>
-    <t xml:space="preserve">33m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">41m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9m</t>
+    <t xml:space="preserve">18m</t>
   </si>
   <si>
     <t xml:space="preserve">29m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">36m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31m</t>
   </si>
   <si>
     <t xml:space="preserve">30m</t>
@@ -303,16 +306,19 @@
     <t xml:space="preserve">46m</t>
   </si>
   <si>
-    <t xml:space="preserve">52m</t>
+    <t xml:space="preserve">36m</t>
   </si>
   <si>
-    <t xml:space="preserve">56m</t>
+    <t xml:space="preserve">39m</t>
   </si>
   <si>
-    <t xml:space="preserve">51m</t>
+    <t xml:space="preserve">50m</t>
   </si>
   <si>
-    <t xml:space="preserve">48m</t>
+    <t xml:space="preserve">35m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28m</t>
   </si>
 </sst>
 </file>
@@ -47640,7 +47646,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>43831</v>
+        <v>43922</v>
       </c>
       <c r="C2" t="s">
         <v>60</v>
@@ -47660,7 +47666,7 @@
         <v>42</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>43831</v>
+        <v>43922</v>
       </c>
       <c r="C3" t="s">
         <v>60</v>
@@ -47680,7 +47686,7 @@
         <v>41</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C4" t="s">
         <v>65</v>
@@ -47700,7 +47706,7 @@
         <v>41</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C5" t="s">
         <v>65</v>
@@ -47720,7 +47726,7 @@
         <v>40</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="C6" t="s">
         <v>68</v>
@@ -47740,7 +47746,7 @@
         <v>40</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="C7" t="s">
         <v>68</v>
@@ -47772,7 +47778,7 @@
         <v>45597</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9">
@@ -47812,7 +47818,7 @@
         <v>45689</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11">
@@ -47880,7 +47886,7 @@
         <v>35</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="C14" t="s">
         <v>65</v>
@@ -47900,7 +47906,7 @@
         <v>35</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="C15" t="s">
         <v>65</v>
@@ -47960,7 +47966,7 @@
         <v>33</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>43831</v>
+        <v>43983</v>
       </c>
       <c r="C18" t="s">
         <v>60</v>
@@ -47980,7 +47986,7 @@
         <v>33</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>43831</v>
+        <v>43983</v>
       </c>
       <c r="C19" t="s">
         <v>60</v>
@@ -48000,7 +48006,7 @@
         <v>32</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C20" t="s">
         <v>60</v>
@@ -48020,7 +48026,7 @@
         <v>32</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C21" t="s">
         <v>60</v>
@@ -48032,7 +48038,7 @@
         <v>44835</v>
       </c>
       <c r="F21" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22">
@@ -48040,7 +48046,7 @@
         <v>31</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>43831</v>
+        <v>43922</v>
       </c>
       <c r="C22" t="s">
         <v>60</v>
@@ -48052,7 +48058,7 @@
         <v>44682</v>
       </c>
       <c r="F22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23">
@@ -48060,7 +48066,7 @@
         <v>31</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>43831</v>
+        <v>43922</v>
       </c>
       <c r="C23" t="s">
         <v>60</v>
@@ -48080,7 +48086,7 @@
         <v>30</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="C24" t="s">
         <v>60</v>
@@ -48100,7 +48106,7 @@
         <v>30</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="C25" t="s">
         <v>60</v>
@@ -48152,7 +48158,7 @@
         <v>44805</v>
       </c>
       <c r="F27" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28">
@@ -48160,7 +48166,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>43831</v>
+        <v>44378</v>
       </c>
       <c r="C28" t="s">
         <v>60</v>
@@ -48172,7 +48178,7 @@
         <v>44713</v>
       </c>
       <c r="F28" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29">
@@ -48180,7 +48186,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>43831</v>
+        <v>44378</v>
       </c>
       <c r="C29" t="s">
         <v>60</v>
@@ -48192,7 +48198,7 @@
         <v>44927</v>
       </c>
       <c r="F29" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30">
@@ -48200,7 +48206,7 @@
         <v>26</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C30" t="s">
         <v>65</v>
@@ -48212,7 +48218,7 @@
         <v>44774</v>
       </c>
       <c r="F30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31">
@@ -48220,7 +48226,7 @@
         <v>26</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C31" t="s">
         <v>65</v>
@@ -48252,7 +48258,7 @@
         <v>44743</v>
       </c>
       <c r="F32" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33">
@@ -48272,7 +48278,7 @@
         <v>45474</v>
       </c>
       <c r="F33" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34">
@@ -48292,7 +48298,7 @@
         <v>45231</v>
       </c>
       <c r="F34" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35">
@@ -48332,7 +48338,7 @@
         <v>44927</v>
       </c>
       <c r="F36" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37">
@@ -48352,7 +48358,7 @@
         <v>45689</v>
       </c>
       <c r="F37" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38">
@@ -48360,7 +48366,7 @@
         <v>21</v>
       </c>
       <c r="B38" s="1" t="n">
-        <v>43831</v>
+        <v>43952</v>
       </c>
       <c r="C38" t="s">
         <v>68</v>
@@ -48380,7 +48386,7 @@
         <v>21</v>
       </c>
       <c r="B39" s="1" t="n">
-        <v>43831</v>
+        <v>43952</v>
       </c>
       <c r="C39" t="s">
         <v>68</v>
@@ -48400,7 +48406,7 @@
         <v>20</v>
       </c>
       <c r="B40" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C40" t="s">
         <v>60</v>
@@ -48412,7 +48418,7 @@
         <v>45078</v>
       </c>
       <c r="F40" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41">
@@ -48420,7 +48426,7 @@
         <v>20</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C41" t="s">
         <v>60</v>
@@ -48432,7 +48438,7 @@
         <v>45413</v>
       </c>
       <c r="F41" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="42">
@@ -48440,7 +48446,7 @@
         <v>19</v>
       </c>
       <c r="B42" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C42" t="s">
         <v>60</v>
@@ -48460,7 +48466,7 @@
         <v>19</v>
       </c>
       <c r="B43" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C43" t="s">
         <v>60</v>
@@ -48472,7 +48478,7 @@
         <v>45536</v>
       </c>
       <c r="F43" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44">
@@ -48480,7 +48486,7 @@
         <v>18</v>
       </c>
       <c r="B44" s="1" t="n">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="C44" t="s">
         <v>60</v>
@@ -48492,7 +48498,7 @@
         <v>44927</v>
       </c>
       <c r="F44" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45">
@@ -48500,7 +48506,7 @@
         <v>18</v>
       </c>
       <c r="B45" s="1" t="n">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="C45" t="s">
         <v>60</v>
@@ -48512,7 +48518,7 @@
         <v>45383</v>
       </c>
       <c r="F45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46">
@@ -48520,7 +48526,7 @@
         <v>17</v>
       </c>
       <c r="B46" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C46" t="s">
         <v>65</v>
@@ -48532,7 +48538,7 @@
         <v>45292</v>
       </c>
       <c r="F46" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47">
@@ -48540,7 +48546,7 @@
         <v>17</v>
       </c>
       <c r="B47" s="1" t="n">
-        <v>43831</v>
+        <v>43891</v>
       </c>
       <c r="C47" t="s">
         <v>65</v>
@@ -48572,7 +48578,7 @@
         <v>44682</v>
       </c>
       <c r="F48" t="s">
-        <v>76</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49">
@@ -48592,7 +48598,7 @@
         <v>44866</v>
       </c>
       <c r="F49" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>